<commit_message>
Update awareness of change of other peoples thoughts, feelings and actions BCT in bcto.xlsx
</commit_message>
<xml_diff>
--- a/BehaviourChangeTechniques/bcto.xlsx
+++ b/BehaviourChangeTechniques/bcto.xlsx
@@ -3692,45 +3692,45 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>awareness of change of other people's thoughts, feelings and actions BCT</t>
+          <t>awareness of change of other peoples thoughts, feelings and actions BCT</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An &lt;awareness of other people’s thoughts, feelings and actions BCT&gt; that increases awareness of changes in what other people think, do or feel. </t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr"/>
+          <t xml:space="preserve">An &lt;awareness of other peoples thoughts, feelings and actions BCT&gt; that increases awareness of changes in what other people think, do or feel. </t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
           <t>awareness of other peoples thoughts, feelings and actions BCT</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
       <c r="J57" s="2" t="inlineStr">
         <is>
           <t>dynamic norms messaging</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr"/>
-      <c r="M57" s="2" t="inlineStr"/>
-      <c r="N57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
+      <c r="M57" s="2" t="n"/>
+      <c r="N57" s="2" t="n"/>
       <c r="O57" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="P57" s="2" t="inlineStr"/>
-      <c r="Q57" s="2" t="inlineStr"/>
-      <c r="R57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="n"/>
+      <c r="Q57" s="2" t="n"/>
+      <c r="R57" s="2" t="n"/>
       <c r="S57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T57" s="2" t="inlineStr"/>
+      <c r="T57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">

</xml_diff>